<commit_message>
Add complete E2E QA Automation Testing Framework (325 test cases + reports + CI workflow)
</commit_message>
<xml_diff>
--- a/reports/test_results.xlsx
+++ b/reports/test_results.xlsx
@@ -27727,12 +27727,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:09:35</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:09:37</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -27754,12 +27754,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:09:37</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:09:39</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -27781,12 +27781,12 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:09:39</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:09:41</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -27808,12 +27808,12 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:09:41</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:09:43</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -27835,12 +27835,12 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:09:43</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:09:45</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -27862,12 +27862,12 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:09:45</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:09:47</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -27889,12 +27889,12 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:09:47</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:09:49</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -27916,12 +27916,12 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:09:49</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:09:51</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -27943,12 +27943,12 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:09:51</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:09:53</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -27970,12 +27970,12 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:09:53</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:09:55</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -27997,12 +27997,12 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:09:55</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:09:57</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -28024,12 +28024,12 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:09:57</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:09:59</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -28051,12 +28051,12 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:09:59</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:10:01</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -28078,12 +28078,12 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:10:01</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:10:03</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -28105,12 +28105,12 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:10:03</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:10:05</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -28132,12 +28132,12 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:10:05</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:10:07</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -28159,12 +28159,12 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:10:07</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:10:09</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -28186,12 +28186,12 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:10:09</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:10:11</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -28213,12 +28213,12 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:10:11</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:10:13</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -28240,12 +28240,12 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:10:13</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:10:15</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -28267,12 +28267,12 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:10:15</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:10:17</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -28294,12 +28294,12 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:10:17</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:10:19</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -28321,12 +28321,12 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:10:19</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:10:21</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -28348,12 +28348,12 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:10:21</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:10:23</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -28375,12 +28375,12 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:10:23</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>09:25:47</t>
+          <t>11:10:25</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">

</xml_diff>